<commit_message>
Batch 6 reviewed and applied
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/work/batch6/batch6-review.xlsx
+++ b/work/batch6/batch6-review.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maost\AppData\Local\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\[01] Martin\[07] Claude Code\NS2-Spanish-Translation\work\batch6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1E66C2A6-19EF-4E78-BA11-9F6CC0B76514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{354F3C4F-C1B7-45BD-83B1-9E7760B3FAB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{8882D7B3-F332-4197-9B35-B13B9C4F23DE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{8882D7B3-F332-4197-9B35-B13B9C4F23DE}"/>
   </bookViews>
   <sheets>
     <sheet name="How to use" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1798" uniqueCount="988">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2141" uniqueCount="991">
   <si>
     <t>Section</t>
   </si>
@@ -3007,6 +3007,15 @@
   </si>
   <si>
     <t>Flagged left</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Use my Spanish</t>
+  </si>
+  <si>
+    <t>Se desbloquea en Partidas Competitivas</t>
   </si>
 </sst>
 </file>
@@ -3567,7 +3576,7 @@
       </c>
       <c r="B10" s="14">
         <f>COUNTA(Review!J2:J343)</f>
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -3576,7 +3585,7 @@
       </c>
       <c r="B11" s="14">
         <f>ROWS(Review!J2:J343)-COUNTA(Review!J2:J343)</f>
-        <v>342</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -3585,7 +3594,7 @@
       </c>
       <c r="B12" s="14">
         <f>COUNTIFS(Review!G2:G343,"?*",Review!J2:J343,"")</f>
-        <v>21</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3595,7 +3604,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8848DF5-3B9B-4C93-95E8-BF114BFDF30F}">
-  <dimension ref="A1:L343"/>
+  <dimension ref="A1:L1048576"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3612,7 +3621,7 @@
     <col min="12" max="12" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3676,7 +3685,9 @@
         <v>19</v>
       </c>
       <c r="I2" s="4"/>
-      <c r="J2" s="7"/>
+      <c r="J2" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K2" s="8"/>
       <c r="L2" s="8"/>
     </row>
@@ -3700,7 +3711,9 @@
       <c r="G3" s="3"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
-      <c r="J3" s="7"/>
+      <c r="J3" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K3" s="8"/>
       <c r="L3" s="8"/>
     </row>
@@ -3730,7 +3743,9 @@
         <v>28</v>
       </c>
       <c r="I4" s="4"/>
-      <c r="J4" s="7"/>
+      <c r="J4" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K4" s="8"/>
       <c r="L4" s="8"/>
     </row>
@@ -3760,7 +3775,9 @@
         <v>33</v>
       </c>
       <c r="I5" s="4"/>
-      <c r="J5" s="7"/>
+      <c r="J5" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K5" s="8"/>
       <c r="L5" s="8"/>
     </row>
@@ -3786,7 +3803,9 @@
       <c r="G6" s="3"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
-      <c r="J6" s="7"/>
+      <c r="J6" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K6" s="8"/>
       <c r="L6" s="8"/>
     </row>
@@ -3814,7 +3833,9 @@
         <v>41</v>
       </c>
       <c r="I7" s="4"/>
-      <c r="J7" s="7"/>
+      <c r="J7" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K7" s="8"/>
       <c r="L7" s="8"/>
     </row>
@@ -3840,7 +3861,9 @@
       <c r="G8" s="3"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
-      <c r="J8" s="7"/>
+      <c r="J8" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K8" s="8"/>
       <c r="L8" s="8"/>
     </row>
@@ -3864,7 +3887,9 @@
       <c r="G9" s="3"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
-      <c r="J9" s="7"/>
+      <c r="J9" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K9" s="8"/>
       <c r="L9" s="8"/>
     </row>
@@ -3888,7 +3913,9 @@
       <c r="G10" s="3"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
-      <c r="J10" s="7"/>
+      <c r="J10" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K10" s="8"/>
       <c r="L10" s="8"/>
     </row>
@@ -3914,7 +3941,9 @@
       <c r="G11" s="3"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
-      <c r="J11" s="7"/>
+      <c r="J11" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K11" s="8"/>
       <c r="L11" s="8"/>
     </row>
@@ -3944,7 +3973,9 @@
         <v>33</v>
       </c>
       <c r="I12" s="4"/>
-      <c r="J12" s="7"/>
+      <c r="J12" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8"/>
     </row>
@@ -3974,7 +4005,9 @@
         <v>62</v>
       </c>
       <c r="I13" s="4"/>
-      <c r="J13" s="7"/>
+      <c r="J13" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8"/>
     </row>
@@ -4000,7 +4033,9 @@
       <c r="G14" s="3"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="7"/>
+      <c r="J14" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8"/>
     </row>
@@ -4030,7 +4065,9 @@
         <v>70</v>
       </c>
       <c r="I15" s="4"/>
-      <c r="J15" s="7"/>
+      <c r="J15" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8"/>
     </row>
@@ -4054,7 +4091,9 @@
       <c r="G16" s="3"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
-      <c r="J16" s="7"/>
+      <c r="J16" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8"/>
     </row>
@@ -4078,7 +4117,9 @@
       <c r="G17" s="3"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
-      <c r="J17" s="7"/>
+      <c r="J17" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8"/>
     </row>
@@ -4102,7 +4143,9 @@
       <c r="G18" s="3"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
-      <c r="J18" s="7"/>
+      <c r="J18" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8"/>
     </row>
@@ -4128,7 +4171,9 @@
       <c r="G19" s="3"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
-      <c r="J19" s="7"/>
+      <c r="J19" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8"/>
     </row>
@@ -4158,7 +4203,9 @@
         <v>87</v>
       </c>
       <c r="I20" s="4"/>
-      <c r="J20" s="7"/>
+      <c r="J20" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8"/>
     </row>
@@ -4184,7 +4231,9 @@
       <c r="G21" s="3"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
-      <c r="J21" s="7"/>
+      <c r="J21" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8"/>
     </row>
@@ -4208,7 +4257,9 @@
       <c r="G22" s="3"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
-      <c r="J22" s="7"/>
+      <c r="J22" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8"/>
     </row>
@@ -4232,7 +4283,9 @@
       <c r="G23" s="3"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
-      <c r="J23" s="7"/>
+      <c r="J23" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8"/>
     </row>
@@ -4256,7 +4309,9 @@
       <c r="G24" s="3"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
-      <c r="J24" s="7"/>
+      <c r="J24" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8"/>
     </row>
@@ -4280,7 +4335,9 @@
       <c r="G25" s="3"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
-      <c r="J25" s="7"/>
+      <c r="J25" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8"/>
     </row>
@@ -4304,8 +4361,12 @@
       <c r="G26" s="3"/>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="8"/>
+      <c r="J26" s="7" t="s">
+        <v>989</v>
+      </c>
+      <c r="K26" s="12" t="s">
+        <v>990</v>
+      </c>
       <c r="L26" s="8"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
@@ -4328,7 +4389,9 @@
       <c r="G27" s="3"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
-      <c r="J27" s="7"/>
+      <c r="J27" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8"/>
     </row>
@@ -4354,7 +4417,9 @@
       <c r="G28" s="3"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
-      <c r="J28" s="7"/>
+      <c r="J28" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8"/>
     </row>
@@ -4378,7 +4443,9 @@
       <c r="G29" s="3"/>
       <c r="H29" s="4"/>
       <c r="I29" s="4"/>
-      <c r="J29" s="7"/>
+      <c r="J29" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8"/>
     </row>
@@ -4404,7 +4471,9 @@
       <c r="G30" s="3"/>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
-      <c r="J30" s="7"/>
+      <c r="J30" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8"/>
     </row>
@@ -4434,7 +4503,9 @@
         <v>120</v>
       </c>
       <c r="I31" s="4"/>
-      <c r="J31" s="7"/>
+      <c r="J31" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
     </row>
@@ -4458,7 +4529,9 @@
       <c r="G32" s="3"/>
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
-      <c r="J32" s="7"/>
+      <c r="J32" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
     </row>
@@ -4484,7 +4557,9 @@
       <c r="I33" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="J33" s="7"/>
+      <c r="J33" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K33" s="8"/>
       <c r="L33" s="8"/>
     </row>
@@ -4512,7 +4587,9 @@
         <v>131</v>
       </c>
       <c r="I34" s="4"/>
-      <c r="J34" s="7"/>
+      <c r="J34" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
     </row>
@@ -4536,7 +4613,9 @@
       <c r="G35" s="3"/>
       <c r="H35" s="4"/>
       <c r="I35" s="4"/>
-      <c r="J35" s="7"/>
+      <c r="J35" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
     </row>
@@ -4560,7 +4639,9 @@
       <c r="G36" s="3"/>
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
-      <c r="J36" s="7"/>
+      <c r="J36" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K36" s="8"/>
       <c r="L36" s="8"/>
     </row>
@@ -4584,7 +4665,9 @@
       <c r="G37" s="3"/>
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
-      <c r="J37" s="7"/>
+      <c r="J37" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K37" s="8"/>
       <c r="L37" s="8"/>
     </row>
@@ -4608,7 +4691,9 @@
       <c r="G38" s="3"/>
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
-      <c r="J38" s="7"/>
+      <c r="J38" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K38" s="8"/>
       <c r="L38" s="8"/>
     </row>
@@ -4632,7 +4717,9 @@
       <c r="G39" s="3"/>
       <c r="H39" s="4"/>
       <c r="I39" s="4"/>
-      <c r="J39" s="7"/>
+      <c r="J39" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K39" s="8"/>
       <c r="L39" s="8"/>
     </row>
@@ -4656,7 +4743,9 @@
       <c r="G40" s="3"/>
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
-      <c r="J40" s="7"/>
+      <c r="J40" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K40" s="8"/>
       <c r="L40" s="8"/>
     </row>
@@ -4680,7 +4769,9 @@
       <c r="G41" s="3"/>
       <c r="H41" s="4"/>
       <c r="I41" s="4"/>
-      <c r="J41" s="7"/>
+      <c r="J41" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K41" s="8"/>
       <c r="L41" s="8"/>
     </row>
@@ -4704,7 +4795,9 @@
       <c r="G42" s="3"/>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
-      <c r="J42" s="7"/>
+      <c r="J42" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K42" s="8"/>
       <c r="L42" s="8"/>
     </row>
@@ -4728,7 +4821,9 @@
       <c r="G43" s="3"/>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
-      <c r="J43" s="7"/>
+      <c r="J43" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K43" s="8"/>
       <c r="L43" s="8"/>
     </row>
@@ -4752,7 +4847,9 @@
       <c r="G44" s="3"/>
       <c r="H44" s="4"/>
       <c r="I44" s="4"/>
-      <c r="J44" s="7"/>
+      <c r="J44" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K44" s="8"/>
       <c r="L44" s="8"/>
     </row>
@@ -4776,7 +4873,9 @@
       <c r="G45" s="3"/>
       <c r="H45" s="4"/>
       <c r="I45" s="4"/>
-      <c r="J45" s="7"/>
+      <c r="J45" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K45" s="8"/>
       <c r="L45" s="8"/>
     </row>
@@ -4800,7 +4899,9 @@
       <c r="G46" s="3"/>
       <c r="H46" s="4"/>
       <c r="I46" s="4"/>
-      <c r="J46" s="7"/>
+      <c r="J46" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K46" s="8"/>
       <c r="L46" s="8"/>
     </row>
@@ -4824,7 +4925,9 @@
       <c r="G47" s="3"/>
       <c r="H47" s="4"/>
       <c r="I47" s="4"/>
-      <c r="J47" s="7"/>
+      <c r="J47" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K47" s="8"/>
       <c r="L47" s="8"/>
     </row>
@@ -4848,7 +4951,9 @@
       <c r="G48" s="3"/>
       <c r="H48" s="4"/>
       <c r="I48" s="4"/>
-      <c r="J48" s="7"/>
+      <c r="J48" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K48" s="8"/>
       <c r="L48" s="8"/>
     </row>
@@ -4872,7 +4977,9 @@
       <c r="G49" s="3"/>
       <c r="H49" s="4"/>
       <c r="I49" s="4"/>
-      <c r="J49" s="7"/>
+      <c r="J49" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K49" s="8"/>
       <c r="L49" s="8"/>
     </row>
@@ -4896,7 +5003,9 @@
       <c r="G50" s="3"/>
       <c r="H50" s="4"/>
       <c r="I50" s="4"/>
-      <c r="J50" s="7"/>
+      <c r="J50" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K50" s="8"/>
       <c r="L50" s="8"/>
     </row>
@@ -4920,7 +5029,9 @@
       <c r="G51" s="3"/>
       <c r="H51" s="4"/>
       <c r="I51" s="4"/>
-      <c r="J51" s="7"/>
+      <c r="J51" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K51" s="8"/>
       <c r="L51" s="8"/>
     </row>
@@ -4944,7 +5055,9 @@
       <c r="G52" s="3"/>
       <c r="H52" s="4"/>
       <c r="I52" s="4"/>
-      <c r="J52" s="7"/>
+      <c r="J52" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K52" s="8"/>
       <c r="L52" s="8"/>
     </row>
@@ -4968,7 +5081,9 @@
       <c r="G53" s="3"/>
       <c r="H53" s="4"/>
       <c r="I53" s="4"/>
-      <c r="J53" s="7"/>
+      <c r="J53" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K53" s="8"/>
       <c r="L53" s="8"/>
     </row>
@@ -4992,7 +5107,9 @@
       <c r="G54" s="3"/>
       <c r="H54" s="4"/>
       <c r="I54" s="4"/>
-      <c r="J54" s="7"/>
+      <c r="J54" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K54" s="8"/>
       <c r="L54" s="8"/>
     </row>
@@ -5016,7 +5133,9 @@
       <c r="G55" s="3"/>
       <c r="H55" s="4"/>
       <c r="I55" s="4"/>
-      <c r="J55" s="7"/>
+      <c r="J55" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K55" s="8"/>
       <c r="L55" s="8"/>
     </row>
@@ -5040,7 +5159,9 @@
       <c r="G56" s="3"/>
       <c r="H56" s="4"/>
       <c r="I56" s="4"/>
-      <c r="J56" s="7"/>
+      <c r="J56" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K56" s="8"/>
       <c r="L56" s="8"/>
     </row>
@@ -5066,7 +5187,9 @@
       <c r="I57" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="J57" s="7"/>
+      <c r="J57" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K57" s="8"/>
       <c r="L57" s="8"/>
     </row>
@@ -5090,7 +5213,9 @@
       <c r="G58" s="3"/>
       <c r="H58" s="4"/>
       <c r="I58" s="4"/>
-      <c r="J58" s="7"/>
+      <c r="J58" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K58" s="8"/>
       <c r="L58" s="8"/>
     </row>
@@ -5114,7 +5239,9 @@
       <c r="G59" s="3"/>
       <c r="H59" s="4"/>
       <c r="I59" s="4"/>
-      <c r="J59" s="7"/>
+      <c r="J59" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K59" s="8"/>
       <c r="L59" s="8"/>
     </row>
@@ -5138,7 +5265,9 @@
       <c r="G60" s="3"/>
       <c r="H60" s="4"/>
       <c r="I60" s="4"/>
-      <c r="J60" s="7"/>
+      <c r="J60" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K60" s="8"/>
       <c r="L60" s="8"/>
     </row>
@@ -5162,7 +5291,9 @@
       <c r="G61" s="3"/>
       <c r="H61" s="4"/>
       <c r="I61" s="4"/>
-      <c r="J61" s="7"/>
+      <c r="J61" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K61" s="8"/>
       <c r="L61" s="8"/>
     </row>
@@ -5186,7 +5317,9 @@
       <c r="G62" s="3"/>
       <c r="H62" s="4"/>
       <c r="I62" s="4"/>
-      <c r="J62" s="7"/>
+      <c r="J62" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K62" s="8"/>
       <c r="L62" s="8"/>
     </row>
@@ -5210,7 +5343,9 @@
       <c r="G63" s="3"/>
       <c r="H63" s="4"/>
       <c r="I63" s="4"/>
-      <c r="J63" s="7"/>
+      <c r="J63" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K63" s="8"/>
       <c r="L63" s="8"/>
     </row>
@@ -5238,7 +5373,9 @@
         <v>222</v>
       </c>
       <c r="I64" s="4"/>
-      <c r="J64" s="7"/>
+      <c r="J64" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K64" s="8"/>
       <c r="L64" s="8"/>
     </row>
@@ -5264,7 +5401,9 @@
       <c r="G65" s="3"/>
       <c r="H65" s="4"/>
       <c r="I65" s="4"/>
-      <c r="J65" s="7"/>
+      <c r="J65" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K65" s="8"/>
       <c r="L65" s="8"/>
     </row>
@@ -5288,7 +5427,9 @@
       <c r="G66" s="3"/>
       <c r="H66" s="4"/>
       <c r="I66" s="4"/>
-      <c r="J66" s="7"/>
+      <c r="J66" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K66" s="8"/>
       <c r="L66" s="8"/>
     </row>
@@ -5312,7 +5453,9 @@
       <c r="G67" s="3"/>
       <c r="H67" s="4"/>
       <c r="I67" s="4"/>
-      <c r="J67" s="7"/>
+      <c r="J67" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K67" s="8"/>
       <c r="L67" s="8"/>
     </row>
@@ -5340,7 +5483,9 @@
         <v>233</v>
       </c>
       <c r="I68" s="4"/>
-      <c r="J68" s="7"/>
+      <c r="J68" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K68" s="8"/>
       <c r="L68" s="8"/>
     </row>
@@ -5364,7 +5509,9 @@
       <c r="G69" s="3"/>
       <c r="H69" s="4"/>
       <c r="I69" s="4"/>
-      <c r="J69" s="7"/>
+      <c r="J69" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K69" s="8"/>
       <c r="L69" s="8"/>
     </row>
@@ -5388,7 +5535,9 @@
       <c r="G70" s="3"/>
       <c r="H70" s="4"/>
       <c r="I70" s="4"/>
-      <c r="J70" s="7"/>
+      <c r="J70" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K70" s="8"/>
       <c r="L70" s="8"/>
     </row>
@@ -5412,7 +5561,9 @@
       <c r="G71" s="3"/>
       <c r="H71" s="4"/>
       <c r="I71" s="4"/>
-      <c r="J71" s="7"/>
+      <c r="J71" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K71" s="8"/>
       <c r="L71" s="8"/>
     </row>
@@ -5436,7 +5587,9 @@
       <c r="G72" s="3"/>
       <c r="H72" s="4"/>
       <c r="I72" s="4"/>
-      <c r="J72" s="7"/>
+      <c r="J72" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K72" s="8"/>
       <c r="L72" s="8"/>
     </row>
@@ -5460,7 +5613,9 @@
       <c r="G73" s="3"/>
       <c r="H73" s="4"/>
       <c r="I73" s="4"/>
-      <c r="J73" s="7"/>
+      <c r="J73" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K73" s="8"/>
       <c r="L73" s="8"/>
     </row>
@@ -5484,7 +5639,9 @@
       <c r="G74" s="3"/>
       <c r="H74" s="4"/>
       <c r="I74" s="4"/>
-      <c r="J74" s="7"/>
+      <c r="J74" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K74" s="8"/>
       <c r="L74" s="8"/>
     </row>
@@ -5510,7 +5667,9 @@
       <c r="I75" s="10" t="s">
         <v>251</v>
       </c>
-      <c r="J75" s="7"/>
+      <c r="J75" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K75" s="8"/>
       <c r="L75" s="8"/>
     </row>
@@ -5534,7 +5693,9 @@
       <c r="G76" s="3"/>
       <c r="H76" s="4"/>
       <c r="I76" s="4"/>
-      <c r="J76" s="7"/>
+      <c r="J76" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K76" s="8"/>
       <c r="L76" s="8"/>
     </row>
@@ -5558,7 +5719,9 @@
       <c r="G77" s="3"/>
       <c r="H77" s="4"/>
       <c r="I77" s="4"/>
-      <c r="J77" s="7"/>
+      <c r="J77" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K77" s="8"/>
       <c r="L77" s="8"/>
     </row>
@@ -5582,7 +5745,9 @@
       <c r="G78" s="3"/>
       <c r="H78" s="4"/>
       <c r="I78" s="4"/>
-      <c r="J78" s="7"/>
+      <c r="J78" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K78" s="8"/>
       <c r="L78" s="8"/>
     </row>
@@ -5606,7 +5771,9 @@
       <c r="G79" s="3"/>
       <c r="H79" s="4"/>
       <c r="I79" s="4"/>
-      <c r="J79" s="7"/>
+      <c r="J79" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K79" s="8"/>
       <c r="L79" s="8"/>
     </row>
@@ -5630,7 +5797,9 @@
       <c r="G80" s="3"/>
       <c r="H80" s="4"/>
       <c r="I80" s="4"/>
-      <c r="J80" s="7"/>
+      <c r="J80" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K80" s="8"/>
       <c r="L80" s="8"/>
     </row>
@@ -5654,7 +5823,9 @@
       <c r="G81" s="3"/>
       <c r="H81" s="4"/>
       <c r="I81" s="4"/>
-      <c r="J81" s="7"/>
+      <c r="J81" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K81" s="8"/>
       <c r="L81" s="8"/>
     </row>
@@ -5678,7 +5849,9 @@
       <c r="G82" s="3"/>
       <c r="H82" s="4"/>
       <c r="I82" s="4"/>
-      <c r="J82" s="7"/>
+      <c r="J82" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K82" s="8"/>
       <c r="L82" s="8"/>
     </row>
@@ -5702,7 +5875,9 @@
       <c r="G83" s="3"/>
       <c r="H83" s="4"/>
       <c r="I83" s="4"/>
-      <c r="J83" s="7"/>
+      <c r="J83" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K83" s="8"/>
       <c r="L83" s="8"/>
     </row>
@@ -5726,7 +5901,9 @@
       <c r="G84" s="3"/>
       <c r="H84" s="4"/>
       <c r="I84" s="4"/>
-      <c r="J84" s="7"/>
+      <c r="J84" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K84" s="8"/>
       <c r="L84" s="8"/>
     </row>
@@ -5750,7 +5927,9 @@
       <c r="G85" s="3"/>
       <c r="H85" s="4"/>
       <c r="I85" s="4"/>
-      <c r="J85" s="7"/>
+      <c r="J85" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K85" s="8"/>
       <c r="L85" s="8"/>
     </row>
@@ -5774,7 +5953,9 @@
       <c r="G86" s="3"/>
       <c r="H86" s="4"/>
       <c r="I86" s="4"/>
-      <c r="J86" s="7"/>
+      <c r="J86" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K86" s="8"/>
       <c r="L86" s="8"/>
     </row>
@@ -5798,7 +5979,9 @@
       <c r="G87" s="3"/>
       <c r="H87" s="4"/>
       <c r="I87" s="4"/>
-      <c r="J87" s="7"/>
+      <c r="J87" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K87" s="8"/>
       <c r="L87" s="8"/>
     </row>
@@ -5822,7 +6005,9 @@
       <c r="G88" s="3"/>
       <c r="H88" s="4"/>
       <c r="I88" s="4"/>
-      <c r="J88" s="7"/>
+      <c r="J88" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K88" s="8"/>
       <c r="L88" s="8"/>
     </row>
@@ -5846,7 +6031,9 @@
       <c r="G89" s="3"/>
       <c r="H89" s="4"/>
       <c r="I89" s="4"/>
-      <c r="J89" s="7"/>
+      <c r="J89" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K89" s="8"/>
       <c r="L89" s="8"/>
     </row>
@@ -5870,7 +6057,9 @@
       <c r="G90" s="3"/>
       <c r="H90" s="4"/>
       <c r="I90" s="4"/>
-      <c r="J90" s="7"/>
+      <c r="J90" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K90" s="8"/>
       <c r="L90" s="8"/>
     </row>
@@ -5898,7 +6087,9 @@
         <v>300</v>
       </c>
       <c r="I91" s="4"/>
-      <c r="J91" s="7"/>
+      <c r="J91" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K91" s="8"/>
       <c r="L91" s="8"/>
     </row>
@@ -5922,7 +6113,9 @@
       <c r="G92" s="3"/>
       <c r="H92" s="4"/>
       <c r="I92" s="4"/>
-      <c r="J92" s="7"/>
+      <c r="J92" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K92" s="8"/>
       <c r="L92" s="8"/>
     </row>
@@ -5946,7 +6139,9 @@
       <c r="G93" s="3"/>
       <c r="H93" s="4"/>
       <c r="I93" s="4"/>
-      <c r="J93" s="7"/>
+      <c r="J93" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K93" s="8"/>
       <c r="L93" s="8"/>
     </row>
@@ -5970,7 +6165,9 @@
       <c r="G94" s="3"/>
       <c r="H94" s="4"/>
       <c r="I94" s="4"/>
-      <c r="J94" s="7"/>
+      <c r="J94" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K94" s="8"/>
       <c r="L94" s="8"/>
     </row>
@@ -5994,7 +6191,9 @@
       <c r="G95" s="3"/>
       <c r="H95" s="4"/>
       <c r="I95" s="4"/>
-      <c r="J95" s="7"/>
+      <c r="J95" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K95" s="8"/>
       <c r="L95" s="8"/>
     </row>
@@ -6018,7 +6217,9 @@
       <c r="G96" s="3"/>
       <c r="H96" s="4"/>
       <c r="I96" s="4"/>
-      <c r="J96" s="7"/>
+      <c r="J96" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K96" s="8"/>
       <c r="L96" s="8"/>
     </row>
@@ -6042,7 +6243,9 @@
       <c r="G97" s="3"/>
       <c r="H97" s="4"/>
       <c r="I97" s="4"/>
-      <c r="J97" s="7"/>
+      <c r="J97" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K97" s="8"/>
       <c r="L97" s="8"/>
     </row>
@@ -6066,7 +6269,9 @@
       <c r="G98" s="3"/>
       <c r="H98" s="4"/>
       <c r="I98" s="4"/>
-      <c r="J98" s="7"/>
+      <c r="J98" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K98" s="8"/>
       <c r="L98" s="8"/>
     </row>
@@ -6096,7 +6301,9 @@
       <c r="I99" s="10" t="s">
         <v>327</v>
       </c>
-      <c r="J99" s="7"/>
+      <c r="J99" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K99" s="8"/>
       <c r="L99" s="8"/>
     </row>
@@ -6120,7 +6327,9 @@
       <c r="G100" s="3"/>
       <c r="H100" s="4"/>
       <c r="I100" s="4"/>
-      <c r="J100" s="7"/>
+      <c r="J100" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K100" s="8"/>
       <c r="L100" s="8"/>
     </row>
@@ -6146,7 +6355,9 @@
       <c r="I101" s="10" t="s">
         <v>327</v>
       </c>
-      <c r="J101" s="7"/>
+      <c r="J101" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K101" s="8"/>
       <c r="L101" s="8"/>
     </row>
@@ -6170,7 +6381,9 @@
       <c r="G102" s="3"/>
       <c r="H102" s="4"/>
       <c r="I102" s="4"/>
-      <c r="J102" s="7"/>
+      <c r="J102" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K102" s="8"/>
       <c r="L102" s="8"/>
     </row>
@@ -6194,7 +6407,9 @@
       <c r="G103" s="3"/>
       <c r="H103" s="4"/>
       <c r="I103" s="4"/>
-      <c r="J103" s="7"/>
+      <c r="J103" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K103" s="8"/>
       <c r="L103" s="8"/>
     </row>
@@ -6218,7 +6433,9 @@
       <c r="G104" s="3"/>
       <c r="H104" s="4"/>
       <c r="I104" s="4"/>
-      <c r="J104" s="7"/>
+      <c r="J104" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K104" s="8"/>
       <c r="L104" s="8"/>
     </row>
@@ -6242,7 +6459,9 @@
       <c r="G105" s="3"/>
       <c r="H105" s="4"/>
       <c r="I105" s="4"/>
-      <c r="J105" s="7"/>
+      <c r="J105" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K105" s="8"/>
       <c r="L105" s="8"/>
     </row>
@@ -6266,7 +6485,9 @@
       <c r="G106" s="3"/>
       <c r="H106" s="4"/>
       <c r="I106" s="4"/>
-      <c r="J106" s="7"/>
+      <c r="J106" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K106" s="8"/>
       <c r="L106" s="8"/>
     </row>
@@ -6290,7 +6511,9 @@
       <c r="G107" s="3"/>
       <c r="H107" s="4"/>
       <c r="I107" s="4"/>
-      <c r="J107" s="7"/>
+      <c r="J107" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K107" s="8"/>
       <c r="L107" s="8"/>
     </row>
@@ -6314,7 +6537,9 @@
       <c r="G108" s="3"/>
       <c r="H108" s="4"/>
       <c r="I108" s="4"/>
-      <c r="J108" s="7"/>
+      <c r="J108" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K108" s="8"/>
       <c r="L108" s="8"/>
     </row>
@@ -6338,7 +6563,9 @@
       <c r="G109" s="3"/>
       <c r="H109" s="4"/>
       <c r="I109" s="4"/>
-      <c r="J109" s="7"/>
+      <c r="J109" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K109" s="8"/>
       <c r="L109" s="8"/>
     </row>
@@ -6362,7 +6589,9 @@
       <c r="G110" s="3"/>
       <c r="H110" s="4"/>
       <c r="I110" s="4"/>
-      <c r="J110" s="7"/>
+      <c r="J110" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K110" s="8"/>
       <c r="L110" s="8"/>
     </row>
@@ -6386,7 +6615,9 @@
       <c r="G111" s="3"/>
       <c r="H111" s="4"/>
       <c r="I111" s="4"/>
-      <c r="J111" s="7"/>
+      <c r="J111" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K111" s="8"/>
       <c r="L111" s="8"/>
     </row>
@@ -6410,7 +6641,9 @@
       <c r="G112" s="3"/>
       <c r="H112" s="4"/>
       <c r="I112" s="4"/>
-      <c r="J112" s="7"/>
+      <c r="J112" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K112" s="8"/>
       <c r="L112" s="8"/>
     </row>
@@ -6434,7 +6667,9 @@
       <c r="G113" s="3"/>
       <c r="H113" s="4"/>
       <c r="I113" s="4"/>
-      <c r="J113" s="7"/>
+      <c r="J113" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K113" s="8"/>
       <c r="L113" s="8"/>
     </row>
@@ -6458,7 +6693,9 @@
       <c r="G114" s="3"/>
       <c r="H114" s="4"/>
       <c r="I114" s="4"/>
-      <c r="J114" s="7"/>
+      <c r="J114" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K114" s="8"/>
       <c r="L114" s="8"/>
     </row>
@@ -6482,7 +6719,9 @@
       <c r="G115" s="3"/>
       <c r="H115" s="4"/>
       <c r="I115" s="4"/>
-      <c r="J115" s="7"/>
+      <c r="J115" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K115" s="8"/>
       <c r="L115" s="8"/>
     </row>
@@ -6506,7 +6745,9 @@
       <c r="G116" s="3"/>
       <c r="H116" s="4"/>
       <c r="I116" s="4"/>
-      <c r="J116" s="7"/>
+      <c r="J116" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K116" s="8"/>
       <c r="L116" s="8"/>
     </row>
@@ -6534,7 +6775,9 @@
         <v>370</v>
       </c>
       <c r="I117" s="4"/>
-      <c r="J117" s="7"/>
+      <c r="J117" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K117" s="8"/>
       <c r="L117" s="8"/>
     </row>
@@ -6558,7 +6801,9 @@
       <c r="G118" s="3"/>
       <c r="H118" s="4"/>
       <c r="I118" s="4"/>
-      <c r="J118" s="7"/>
+      <c r="J118" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K118" s="8"/>
       <c r="L118" s="8"/>
     </row>
@@ -6582,7 +6827,9 @@
       <c r="G119" s="3"/>
       <c r="H119" s="4"/>
       <c r="I119" s="4"/>
-      <c r="J119" s="7"/>
+      <c r="J119" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K119" s="8"/>
       <c r="L119" s="8"/>
     </row>
@@ -6606,7 +6853,9 @@
       <c r="G120" s="3"/>
       <c r="H120" s="4"/>
       <c r="I120" s="4"/>
-      <c r="J120" s="7"/>
+      <c r="J120" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K120" s="8"/>
       <c r="L120" s="8"/>
     </row>
@@ -6630,7 +6879,9 @@
       <c r="G121" s="3"/>
       <c r="H121" s="4"/>
       <c r="I121" s="4"/>
-      <c r="J121" s="7"/>
+      <c r="J121" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K121" s="8"/>
       <c r="L121" s="8"/>
     </row>
@@ -6654,7 +6905,9 @@
       <c r="G122" s="3"/>
       <c r="H122" s="4"/>
       <c r="I122" s="4"/>
-      <c r="J122" s="7"/>
+      <c r="J122" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K122" s="8"/>
       <c r="L122" s="8"/>
     </row>
@@ -6678,7 +6931,9 @@
       <c r="G123" s="3"/>
       <c r="H123" s="4"/>
       <c r="I123" s="4"/>
-      <c r="J123" s="7"/>
+      <c r="J123" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K123" s="8"/>
       <c r="L123" s="8"/>
     </row>
@@ -6702,7 +6957,9 @@
       <c r="G124" s="3"/>
       <c r="H124" s="4"/>
       <c r="I124" s="4"/>
-      <c r="J124" s="7"/>
+      <c r="J124" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K124" s="8"/>
       <c r="L124" s="8"/>
     </row>
@@ -6726,7 +6983,9 @@
       <c r="G125" s="3"/>
       <c r="H125" s="4"/>
       <c r="I125" s="4"/>
-      <c r="J125" s="7"/>
+      <c r="J125" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K125" s="8"/>
       <c r="L125" s="8"/>
     </row>
@@ -6750,7 +7009,9 @@
       <c r="G126" s="3"/>
       <c r="H126" s="4"/>
       <c r="I126" s="4"/>
-      <c r="J126" s="7"/>
+      <c r="J126" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K126" s="8"/>
       <c r="L126" s="8"/>
     </row>
@@ -6774,7 +7035,9 @@
       <c r="G127" s="3"/>
       <c r="H127" s="4"/>
       <c r="I127" s="4"/>
-      <c r="J127" s="7"/>
+      <c r="J127" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K127" s="8"/>
       <c r="L127" s="8"/>
     </row>
@@ -6798,7 +7061,9 @@
       <c r="G128" s="3"/>
       <c r="H128" s="4"/>
       <c r="I128" s="4"/>
-      <c r="J128" s="7"/>
+      <c r="J128" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K128" s="8"/>
       <c r="L128" s="8"/>
     </row>
@@ -6822,7 +7087,9 @@
       <c r="G129" s="3"/>
       <c r="H129" s="4"/>
       <c r="I129" s="4"/>
-      <c r="J129" s="7"/>
+      <c r="J129" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K129" s="8"/>
       <c r="L129" s="8"/>
     </row>
@@ -6846,7 +7113,9 @@
       <c r="G130" s="3"/>
       <c r="H130" s="4"/>
       <c r="I130" s="4"/>
-      <c r="J130" s="7"/>
+      <c r="J130" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K130" s="8"/>
       <c r="L130" s="8"/>
     </row>
@@ -6870,7 +7139,9 @@
       <c r="G131" s="3"/>
       <c r="H131" s="4"/>
       <c r="I131" s="4"/>
-      <c r="J131" s="7"/>
+      <c r="J131" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K131" s="8"/>
       <c r="L131" s="8"/>
     </row>
@@ -6894,7 +7165,9 @@
       <c r="G132" s="3"/>
       <c r="H132" s="4"/>
       <c r="I132" s="4"/>
-      <c r="J132" s="7"/>
+      <c r="J132" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K132" s="8"/>
       <c r="L132" s="8"/>
     </row>
@@ -6918,7 +7191,9 @@
       <c r="G133" s="3"/>
       <c r="H133" s="4"/>
       <c r="I133" s="4"/>
-      <c r="J133" s="7"/>
+      <c r="J133" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K133" s="8"/>
       <c r="L133" s="8"/>
     </row>
@@ -6942,7 +7217,9 @@
       <c r="G134" s="3"/>
       <c r="H134" s="4"/>
       <c r="I134" s="4"/>
-      <c r="J134" s="7"/>
+      <c r="J134" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K134" s="8"/>
       <c r="L134" s="8"/>
     </row>
@@ -6968,7 +7245,9 @@
       <c r="I135" s="10" t="s">
         <v>407</v>
       </c>
-      <c r="J135" s="7"/>
+      <c r="J135" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K135" s="8"/>
       <c r="L135" s="8"/>
     </row>
@@ -6992,7 +7271,9 @@
       <c r="G136" s="3"/>
       <c r="H136" s="4"/>
       <c r="I136" s="4"/>
-      <c r="J136" s="7"/>
+      <c r="J136" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K136" s="8"/>
       <c r="L136" s="8"/>
     </row>
@@ -7016,7 +7297,9 @@
       <c r="G137" s="3"/>
       <c r="H137" s="4"/>
       <c r="I137" s="4"/>
-      <c r="J137" s="7"/>
+      <c r="J137" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K137" s="8"/>
       <c r="L137" s="8"/>
     </row>
@@ -7040,7 +7323,9 @@
       <c r="G138" s="3"/>
       <c r="H138" s="4"/>
       <c r="I138" s="4"/>
-      <c r="J138" s="7"/>
+      <c r="J138" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K138" s="8"/>
       <c r="L138" s="8"/>
     </row>
@@ -7064,7 +7349,9 @@
       <c r="G139" s="3"/>
       <c r="H139" s="4"/>
       <c r="I139" s="4"/>
-      <c r="J139" s="7"/>
+      <c r="J139" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K139" s="8"/>
       <c r="L139" s="8"/>
     </row>
@@ -7088,7 +7375,9 @@
       <c r="G140" s="3"/>
       <c r="H140" s="4"/>
       <c r="I140" s="4"/>
-      <c r="J140" s="7"/>
+      <c r="J140" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K140" s="8"/>
       <c r="L140" s="8"/>
     </row>
@@ -7112,7 +7401,9 @@
       <c r="G141" s="3"/>
       <c r="H141" s="4"/>
       <c r="I141" s="4"/>
-      <c r="J141" s="7"/>
+      <c r="J141" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K141" s="8"/>
       <c r="L141" s="8"/>
     </row>
@@ -7136,7 +7427,9 @@
       <c r="G142" s="3"/>
       <c r="H142" s="4"/>
       <c r="I142" s="4"/>
-      <c r="J142" s="7"/>
+      <c r="J142" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K142" s="8"/>
       <c r="L142" s="8"/>
     </row>
@@ -7160,7 +7453,9 @@
       <c r="G143" s="3"/>
       <c r="H143" s="4"/>
       <c r="I143" s="4"/>
-      <c r="J143" s="7"/>
+      <c r="J143" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K143" s="8"/>
       <c r="L143" s="8"/>
     </row>
@@ -7184,7 +7479,9 @@
       <c r="G144" s="3"/>
       <c r="H144" s="4"/>
       <c r="I144" s="4"/>
-      <c r="J144" s="7"/>
+      <c r="J144" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K144" s="8"/>
       <c r="L144" s="8"/>
     </row>
@@ -7208,7 +7505,9 @@
       <c r="G145" s="3"/>
       <c r="H145" s="4"/>
       <c r="I145" s="4"/>
-      <c r="J145" s="7"/>
+      <c r="J145" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K145" s="8"/>
       <c r="L145" s="8"/>
     </row>
@@ -7232,7 +7531,9 @@
       <c r="G146" s="3"/>
       <c r="H146" s="4"/>
       <c r="I146" s="4"/>
-      <c r="J146" s="7"/>
+      <c r="J146" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K146" s="8"/>
       <c r="L146" s="8"/>
     </row>
@@ -7258,7 +7559,9 @@
       <c r="I147" s="10" t="s">
         <v>432</v>
       </c>
-      <c r="J147" s="7"/>
+      <c r="J147" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K147" s="8"/>
       <c r="L147" s="8"/>
     </row>
@@ -7282,7 +7585,9 @@
       <c r="G148" s="3"/>
       <c r="H148" s="4"/>
       <c r="I148" s="4"/>
-      <c r="J148" s="7"/>
+      <c r="J148" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K148" s="8"/>
       <c r="L148" s="8"/>
     </row>
@@ -7310,7 +7615,9 @@
         <v>439</v>
       </c>
       <c r="I149" s="4"/>
-      <c r="J149" s="7"/>
+      <c r="J149" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K149" s="8"/>
       <c r="L149" s="8"/>
     </row>
@@ -7334,7 +7641,9 @@
       <c r="G150" s="3"/>
       <c r="H150" s="4"/>
       <c r="I150" s="4"/>
-      <c r="J150" s="7"/>
+      <c r="J150" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K150" s="8"/>
       <c r="L150" s="8"/>
     </row>
@@ -7358,7 +7667,9 @@
       <c r="G151" s="3"/>
       <c r="H151" s="4"/>
       <c r="I151" s="4"/>
-      <c r="J151" s="7"/>
+      <c r="J151" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K151" s="8"/>
       <c r="L151" s="8"/>
     </row>
@@ -7382,7 +7693,9 @@
       <c r="G152" s="3"/>
       <c r="H152" s="4"/>
       <c r="I152" s="4"/>
-      <c r="J152" s="7"/>
+      <c r="J152" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K152" s="8"/>
       <c r="L152" s="8"/>
     </row>
@@ -7406,7 +7719,9 @@
       <c r="G153" s="3"/>
       <c r="H153" s="4"/>
       <c r="I153" s="4"/>
-      <c r="J153" s="7"/>
+      <c r="J153" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K153" s="8"/>
       <c r="L153" s="8"/>
     </row>
@@ -7434,7 +7749,9 @@
         <v>454</v>
       </c>
       <c r="I154" s="4"/>
-      <c r="J154" s="7"/>
+      <c r="J154" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K154" s="8"/>
       <c r="L154" s="8"/>
     </row>
@@ -7458,7 +7775,9 @@
       <c r="G155" s="3"/>
       <c r="H155" s="4"/>
       <c r="I155" s="4"/>
-      <c r="J155" s="7"/>
+      <c r="J155" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K155" s="8"/>
       <c r="L155" s="8"/>
     </row>
@@ -7482,7 +7801,9 @@
       <c r="G156" s="3"/>
       <c r="H156" s="4"/>
       <c r="I156" s="4"/>
-      <c r="J156" s="7"/>
+      <c r="J156" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K156" s="8"/>
       <c r="L156" s="8"/>
     </row>
@@ -7506,7 +7827,9 @@
       <c r="G157" s="3"/>
       <c r="H157" s="4"/>
       <c r="I157" s="4"/>
-      <c r="J157" s="7"/>
+      <c r="J157" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K157" s="8"/>
       <c r="L157" s="8"/>
     </row>
@@ -7530,7 +7853,9 @@
       <c r="G158" s="3"/>
       <c r="H158" s="4"/>
       <c r="I158" s="4"/>
-      <c r="J158" s="7"/>
+      <c r="J158" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K158" s="8"/>
       <c r="L158" s="8"/>
     </row>
@@ -7554,7 +7879,9 @@
       <c r="G159" s="3"/>
       <c r="H159" s="4"/>
       <c r="I159" s="4"/>
-      <c r="J159" s="7"/>
+      <c r="J159" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K159" s="8"/>
       <c r="L159" s="8"/>
     </row>
@@ -7578,7 +7905,9 @@
       <c r="G160" s="3"/>
       <c r="H160" s="4"/>
       <c r="I160" s="4"/>
-      <c r="J160" s="7"/>
+      <c r="J160" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K160" s="8"/>
       <c r="L160" s="8"/>
     </row>
@@ -7604,7 +7933,9 @@
       <c r="I161" s="10" t="s">
         <v>476</v>
       </c>
-      <c r="J161" s="7"/>
+      <c r="J161" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K161" s="8"/>
       <c r="L161" s="8"/>
     </row>
@@ -7628,7 +7959,9 @@
       <c r="G162" s="3"/>
       <c r="H162" s="4"/>
       <c r="I162" s="4"/>
-      <c r="J162" s="7"/>
+      <c r="J162" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K162" s="8"/>
       <c r="L162" s="8"/>
     </row>
@@ -7652,7 +7985,9 @@
       <c r="G163" s="3"/>
       <c r="H163" s="4"/>
       <c r="I163" s="4"/>
-      <c r="J163" s="7"/>
+      <c r="J163" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K163" s="8"/>
       <c r="L163" s="8"/>
     </row>
@@ -7676,7 +8011,9 @@
       <c r="G164" s="3"/>
       <c r="H164" s="4"/>
       <c r="I164" s="4"/>
-      <c r="J164" s="7"/>
+      <c r="J164" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K164" s="8"/>
       <c r="L164" s="8"/>
     </row>
@@ -7700,7 +8037,9 @@
       <c r="G165" s="3"/>
       <c r="H165" s="4"/>
       <c r="I165" s="4"/>
-      <c r="J165" s="7"/>
+      <c r="J165" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K165" s="8"/>
       <c r="L165" s="8"/>
     </row>
@@ -7724,7 +8063,9 @@
       <c r="G166" s="3"/>
       <c r="H166" s="4"/>
       <c r="I166" s="4"/>
-      <c r="J166" s="7"/>
+      <c r="J166" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K166" s="8"/>
       <c r="L166" s="8"/>
     </row>
@@ -7748,7 +8089,9 @@
       <c r="G167" s="3"/>
       <c r="H167" s="4"/>
       <c r="I167" s="4"/>
-      <c r="J167" s="7"/>
+      <c r="J167" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K167" s="8"/>
       <c r="L167" s="8"/>
     </row>
@@ -7772,7 +8115,9 @@
       <c r="G168" s="3"/>
       <c r="H168" s="4"/>
       <c r="I168" s="4"/>
-      <c r="J168" s="7"/>
+      <c r="J168" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K168" s="8"/>
       <c r="L168" s="8"/>
     </row>
@@ -7796,7 +8141,9 @@
       <c r="G169" s="3"/>
       <c r="H169" s="4"/>
       <c r="I169" s="4"/>
-      <c r="J169" s="7"/>
+      <c r="J169" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K169" s="8"/>
       <c r="L169" s="8"/>
     </row>
@@ -7820,7 +8167,9 @@
       <c r="G170" s="3"/>
       <c r="H170" s="4"/>
       <c r="I170" s="4"/>
-      <c r="J170" s="7"/>
+      <c r="J170" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K170" s="8"/>
       <c r="L170" s="8"/>
     </row>
@@ -7848,7 +8197,9 @@
         <v>507</v>
       </c>
       <c r="I171" s="4"/>
-      <c r="J171" s="7"/>
+      <c r="J171" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K171" s="8"/>
       <c r="L171" s="8"/>
     </row>
@@ -7872,7 +8223,9 @@
       <c r="G172" s="3"/>
       <c r="H172" s="4"/>
       <c r="I172" s="4"/>
-      <c r="J172" s="7"/>
+      <c r="J172" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K172" s="8"/>
       <c r="L172" s="8"/>
     </row>
@@ -7896,7 +8249,9 @@
       <c r="G173" s="3"/>
       <c r="H173" s="4"/>
       <c r="I173" s="4"/>
-      <c r="J173" s="7"/>
+      <c r="J173" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K173" s="8"/>
       <c r="L173" s="8"/>
     </row>
@@ -7920,7 +8275,9 @@
       <c r="G174" s="3"/>
       <c r="H174" s="4"/>
       <c r="I174" s="4"/>
-      <c r="J174" s="7"/>
+      <c r="J174" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K174" s="8"/>
       <c r="L174" s="8"/>
     </row>
@@ -7944,7 +8301,9 @@
       <c r="G175" s="3"/>
       <c r="H175" s="4"/>
       <c r="I175" s="4"/>
-      <c r="J175" s="7"/>
+      <c r="J175" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K175" s="8"/>
       <c r="L175" s="8"/>
     </row>
@@ -7968,7 +8327,9 @@
       <c r="G176" s="3"/>
       <c r="H176" s="4"/>
       <c r="I176" s="4"/>
-      <c r="J176" s="7"/>
+      <c r="J176" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K176" s="8"/>
       <c r="L176" s="8"/>
     </row>
@@ -7992,7 +8353,9 @@
       <c r="G177" s="3"/>
       <c r="H177" s="4"/>
       <c r="I177" s="4"/>
-      <c r="J177" s="7"/>
+      <c r="J177" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K177" s="8"/>
       <c r="L177" s="8"/>
     </row>
@@ -8016,7 +8379,9 @@
       <c r="G178" s="3"/>
       <c r="H178" s="4"/>
       <c r="I178" s="4"/>
-      <c r="J178" s="7"/>
+      <c r="J178" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K178" s="8"/>
       <c r="L178" s="8"/>
     </row>
@@ -8044,7 +8409,9 @@
         <v>533</v>
       </c>
       <c r="I179" s="4"/>
-      <c r="J179" s="7"/>
+      <c r="J179" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K179" s="8"/>
       <c r="L179" s="8"/>
     </row>
@@ -8068,7 +8435,9 @@
       <c r="G180" s="3"/>
       <c r="H180" s="4"/>
       <c r="I180" s="4"/>
-      <c r="J180" s="7"/>
+      <c r="J180" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K180" s="8"/>
       <c r="L180" s="8"/>
     </row>
@@ -8092,7 +8461,9 @@
       <c r="G181" s="3"/>
       <c r="H181" s="4"/>
       <c r="I181" s="4"/>
-      <c r="J181" s="7"/>
+      <c r="J181" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K181" s="8"/>
       <c r="L181" s="8"/>
     </row>
@@ -8116,7 +8487,9 @@
       <c r="G182" s="3"/>
       <c r="H182" s="4"/>
       <c r="I182" s="4"/>
-      <c r="J182" s="7"/>
+      <c r="J182" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K182" s="8"/>
       <c r="L182" s="8"/>
     </row>
@@ -8140,7 +8513,9 @@
       <c r="G183" s="3"/>
       <c r="H183" s="4"/>
       <c r="I183" s="4"/>
-      <c r="J183" s="7"/>
+      <c r="J183" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K183" s="8"/>
       <c r="L183" s="8"/>
     </row>
@@ -8164,7 +8539,9 @@
       <c r="G184" s="3"/>
       <c r="H184" s="4"/>
       <c r="I184" s="4"/>
-      <c r="J184" s="7"/>
+      <c r="J184" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K184" s="8"/>
       <c r="L184" s="8"/>
     </row>
@@ -8188,7 +8565,9 @@
       <c r="G185" s="3"/>
       <c r="H185" s="4"/>
       <c r="I185" s="4"/>
-      <c r="J185" s="7"/>
+      <c r="J185" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K185" s="8"/>
       <c r="L185" s="8"/>
     </row>
@@ -8212,7 +8591,9 @@
       <c r="G186" s="3"/>
       <c r="H186" s="4"/>
       <c r="I186" s="4"/>
-      <c r="J186" s="7"/>
+      <c r="J186" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K186" s="8"/>
       <c r="L186" s="8"/>
     </row>
@@ -8236,7 +8617,9 @@
       <c r="G187" s="3"/>
       <c r="H187" s="4"/>
       <c r="I187" s="4"/>
-      <c r="J187" s="7"/>
+      <c r="J187" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K187" s="8"/>
       <c r="L187" s="8"/>
     </row>
@@ -8260,7 +8643,9 @@
       <c r="G188" s="3"/>
       <c r="H188" s="4"/>
       <c r="I188" s="4"/>
-      <c r="J188" s="7"/>
+      <c r="J188" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K188" s="8"/>
       <c r="L188" s="8"/>
     </row>
@@ -8284,7 +8669,9 @@
       <c r="G189" s="3"/>
       <c r="H189" s="4"/>
       <c r="I189" s="4"/>
-      <c r="J189" s="7"/>
+      <c r="J189" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K189" s="8"/>
       <c r="L189" s="8"/>
     </row>
@@ -8308,7 +8695,9 @@
       <c r="G190" s="3"/>
       <c r="H190" s="4"/>
       <c r="I190" s="4"/>
-      <c r="J190" s="7"/>
+      <c r="J190" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K190" s="8"/>
       <c r="L190" s="8"/>
     </row>
@@ -8332,7 +8721,9 @@
       <c r="G191" s="3"/>
       <c r="H191" s="4"/>
       <c r="I191" s="4"/>
-      <c r="J191" s="7"/>
+      <c r="J191" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K191" s="8"/>
       <c r="L191" s="8"/>
     </row>
@@ -8356,7 +8747,9 @@
       <c r="G192" s="3"/>
       <c r="H192" s="4"/>
       <c r="I192" s="4"/>
-      <c r="J192" s="7"/>
+      <c r="J192" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K192" s="8"/>
       <c r="L192" s="8"/>
     </row>
@@ -8380,7 +8773,9 @@
       <c r="G193" s="3"/>
       <c r="H193" s="4"/>
       <c r="I193" s="4"/>
-      <c r="J193" s="7"/>
+      <c r="J193" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K193" s="8"/>
       <c r="L193" s="8"/>
     </row>
@@ -8404,7 +8799,9 @@
       <c r="G194" s="3"/>
       <c r="H194" s="4"/>
       <c r="I194" s="4"/>
-      <c r="J194" s="7"/>
+      <c r="J194" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K194" s="8"/>
       <c r="L194" s="8"/>
     </row>
@@ -8428,7 +8825,9 @@
       <c r="G195" s="3"/>
       <c r="H195" s="4"/>
       <c r="I195" s="4"/>
-      <c r="J195" s="7"/>
+      <c r="J195" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K195" s="8"/>
       <c r="L195" s="8"/>
     </row>
@@ -8452,7 +8851,9 @@
       <c r="G196" s="3"/>
       <c r="H196" s="4"/>
       <c r="I196" s="4"/>
-      <c r="J196" s="7"/>
+      <c r="J196" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K196" s="8"/>
       <c r="L196" s="8"/>
     </row>
@@ -8476,7 +8877,9 @@
       <c r="G197" s="3"/>
       <c r="H197" s="4"/>
       <c r="I197" s="4"/>
-      <c r="J197" s="7"/>
+      <c r="J197" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K197" s="8"/>
       <c r="L197" s="8"/>
     </row>
@@ -8500,7 +8903,9 @@
       <c r="G198" s="3"/>
       <c r="H198" s="4"/>
       <c r="I198" s="4"/>
-      <c r="J198" s="7"/>
+      <c r="J198" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K198" s="8"/>
       <c r="L198" s="8"/>
     </row>
@@ -8524,7 +8929,9 @@
       <c r="G199" s="3"/>
       <c r="H199" s="4"/>
       <c r="I199" s="4"/>
-      <c r="J199" s="7"/>
+      <c r="J199" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K199" s="8"/>
       <c r="L199" s="8"/>
     </row>
@@ -8546,7 +8953,9 @@
       <c r="I200" s="10" t="s">
         <v>595</v>
       </c>
-      <c r="J200" s="7"/>
+      <c r="J200" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K200" s="8"/>
       <c r="L200" s="8"/>
     </row>
@@ -8570,7 +8979,9 @@
       <c r="G201" s="3"/>
       <c r="H201" s="4"/>
       <c r="I201" s="4"/>
-      <c r="J201" s="7"/>
+      <c r="J201" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K201" s="8"/>
       <c r="L201" s="8"/>
     </row>
@@ -8592,7 +9003,9 @@
       <c r="I202" s="10" t="s">
         <v>595</v>
       </c>
-      <c r="J202" s="7"/>
+      <c r="J202" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K202" s="8"/>
       <c r="L202" s="8"/>
     </row>
@@ -8616,7 +9029,9 @@
       <c r="G203" s="3"/>
       <c r="H203" s="4"/>
       <c r="I203" s="4"/>
-      <c r="J203" s="7"/>
+      <c r="J203" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K203" s="8"/>
       <c r="L203" s="8"/>
     </row>
@@ -8638,7 +9053,9 @@
       <c r="I204" s="10" t="s">
         <v>595</v>
       </c>
-      <c r="J204" s="7"/>
+      <c r="J204" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K204" s="8"/>
       <c r="L204" s="8"/>
     </row>
@@ -8662,7 +9079,9 @@
       <c r="G205" s="3"/>
       <c r="H205" s="4"/>
       <c r="I205" s="4"/>
-      <c r="J205" s="7"/>
+      <c r="J205" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K205" s="8"/>
       <c r="L205" s="8"/>
     </row>
@@ -8684,7 +9103,9 @@
       <c r="I206" s="10" t="s">
         <v>595</v>
       </c>
-      <c r="J206" s="7"/>
+      <c r="J206" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K206" s="8"/>
       <c r="L206" s="8"/>
     </row>
@@ -8708,7 +9129,9 @@
       <c r="G207" s="3"/>
       <c r="H207" s="4"/>
       <c r="I207" s="4"/>
-      <c r="J207" s="7"/>
+      <c r="J207" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K207" s="8"/>
       <c r="L207" s="8"/>
     </row>
@@ -8730,7 +9153,9 @@
       <c r="I208" s="10" t="s">
         <v>595</v>
       </c>
-      <c r="J208" s="7"/>
+      <c r="J208" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K208" s="8"/>
       <c r="L208" s="8"/>
     </row>
@@ -8754,7 +9179,9 @@
       <c r="G209" s="3"/>
       <c r="H209" s="4"/>
       <c r="I209" s="4"/>
-      <c r="J209" s="7"/>
+      <c r="J209" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K209" s="8"/>
       <c r="L209" s="8"/>
     </row>
@@ -8776,7 +9203,9 @@
       <c r="I210" s="10" t="s">
         <v>595</v>
       </c>
-      <c r="J210" s="7"/>
+      <c r="J210" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K210" s="8"/>
       <c r="L210" s="8"/>
     </row>
@@ -8800,7 +9229,9 @@
       <c r="G211" s="3"/>
       <c r="H211" s="4"/>
       <c r="I211" s="4"/>
-      <c r="J211" s="7"/>
+      <c r="J211" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K211" s="8"/>
       <c r="L211" s="8"/>
     </row>
@@ -8822,7 +9253,9 @@
       <c r="I212" s="10" t="s">
         <v>595</v>
       </c>
-      <c r="J212" s="7"/>
+      <c r="J212" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K212" s="8"/>
       <c r="L212" s="8"/>
     </row>
@@ -8846,7 +9279,9 @@
       <c r="G213" s="3"/>
       <c r="H213" s="4"/>
       <c r="I213" s="4"/>
-      <c r="J213" s="7"/>
+      <c r="J213" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K213" s="8"/>
       <c r="L213" s="8"/>
     </row>
@@ -8868,7 +9303,9 @@
       <c r="I214" s="10" t="s">
         <v>595</v>
       </c>
-      <c r="J214" s="7"/>
+      <c r="J214" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K214" s="8"/>
       <c r="L214" s="8"/>
     </row>
@@ -8892,7 +9329,9 @@
       <c r="G215" s="3"/>
       <c r="H215" s="4"/>
       <c r="I215" s="4"/>
-      <c r="J215" s="7"/>
+      <c r="J215" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K215" s="8"/>
       <c r="L215" s="8"/>
     </row>
@@ -8916,7 +9355,9 @@
       <c r="G216" s="3"/>
       <c r="H216" s="4"/>
       <c r="I216" s="4"/>
-      <c r="J216" s="7"/>
+      <c r="J216" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K216" s="8"/>
       <c r="L216" s="8"/>
     </row>
@@ -8940,7 +9381,9 @@
       <c r="G217" s="3"/>
       <c r="H217" s="4"/>
       <c r="I217" s="4"/>
-      <c r="J217" s="7"/>
+      <c r="J217" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K217" s="8"/>
       <c r="L217" s="8"/>
     </row>
@@ -8964,7 +9407,9 @@
       <c r="G218" s="3"/>
       <c r="H218" s="4"/>
       <c r="I218" s="4"/>
-      <c r="J218" s="7"/>
+      <c r="J218" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K218" s="8"/>
       <c r="L218" s="8"/>
     </row>
@@ -8988,7 +9433,9 @@
       <c r="G219" s="3"/>
       <c r="H219" s="4"/>
       <c r="I219" s="4"/>
-      <c r="J219" s="7"/>
+      <c r="J219" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K219" s="8"/>
       <c r="L219" s="8"/>
     </row>
@@ -9012,7 +9459,9 @@
       <c r="G220" s="3"/>
       <c r="H220" s="4"/>
       <c r="I220" s="4"/>
-      <c r="J220" s="7"/>
+      <c r="J220" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K220" s="8"/>
       <c r="L220" s="8"/>
     </row>
@@ -9036,7 +9485,9 @@
       <c r="G221" s="3"/>
       <c r="H221" s="4"/>
       <c r="I221" s="4"/>
-      <c r="J221" s="7"/>
+      <c r="J221" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K221" s="8"/>
       <c r="L221" s="8"/>
     </row>
@@ -9060,7 +9511,9 @@
       <c r="G222" s="3"/>
       <c r="H222" s="4"/>
       <c r="I222" s="4"/>
-      <c r="J222" s="7"/>
+      <c r="J222" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K222" s="8"/>
       <c r="L222" s="8"/>
     </row>
@@ -9084,7 +9537,9 @@
       <c r="G223" s="3"/>
       <c r="H223" s="4"/>
       <c r="I223" s="4"/>
-      <c r="J223" s="7"/>
+      <c r="J223" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K223" s="8"/>
       <c r="L223" s="8"/>
     </row>
@@ -9108,7 +9563,9 @@
       <c r="G224" s="3"/>
       <c r="H224" s="4"/>
       <c r="I224" s="4"/>
-      <c r="J224" s="7"/>
+      <c r="J224" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K224" s="8"/>
       <c r="L224" s="8"/>
     </row>
@@ -9132,7 +9589,9 @@
       <c r="G225" s="3"/>
       <c r="H225" s="4"/>
       <c r="I225" s="4"/>
-      <c r="J225" s="7"/>
+      <c r="J225" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K225" s="8"/>
       <c r="L225" s="8"/>
     </row>
@@ -9156,7 +9615,9 @@
       <c r="G226" s="3"/>
       <c r="H226" s="4"/>
       <c r="I226" s="4"/>
-      <c r="J226" s="7"/>
+      <c r="J226" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K226" s="8"/>
       <c r="L226" s="8"/>
     </row>
@@ -9180,7 +9641,9 @@
       <c r="G227" s="3"/>
       <c r="H227" s="4"/>
       <c r="I227" s="4"/>
-      <c r="J227" s="7"/>
+      <c r="J227" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K227" s="8"/>
       <c r="L227" s="8"/>
     </row>
@@ -9204,7 +9667,9 @@
       <c r="G228" s="3"/>
       <c r="H228" s="4"/>
       <c r="I228" s="4"/>
-      <c r="J228" s="7"/>
+      <c r="J228" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K228" s="8"/>
       <c r="L228" s="8"/>
     </row>
@@ -9228,7 +9693,9 @@
       <c r="G229" s="3"/>
       <c r="H229" s="4"/>
       <c r="I229" s="4"/>
-      <c r="J229" s="7"/>
+      <c r="J229" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K229" s="8"/>
       <c r="L229" s="8"/>
     </row>
@@ -9252,7 +9719,9 @@
       <c r="G230" s="3"/>
       <c r="H230" s="4"/>
       <c r="I230" s="4"/>
-      <c r="J230" s="7"/>
+      <c r="J230" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K230" s="8"/>
       <c r="L230" s="8"/>
     </row>
@@ -9276,7 +9745,9 @@
       <c r="G231" s="3"/>
       <c r="H231" s="4"/>
       <c r="I231" s="4"/>
-      <c r="J231" s="7"/>
+      <c r="J231" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K231" s="8"/>
       <c r="L231" s="8"/>
     </row>
@@ -9300,7 +9771,9 @@
       <c r="G232" s="3"/>
       <c r="H232" s="4"/>
       <c r="I232" s="4"/>
-      <c r="J232" s="7"/>
+      <c r="J232" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K232" s="8"/>
       <c r="L232" s="8"/>
     </row>
@@ -9324,7 +9797,9 @@
       <c r="G233" s="3"/>
       <c r="H233" s="4"/>
       <c r="I233" s="4"/>
-      <c r="J233" s="7"/>
+      <c r="J233" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K233" s="8"/>
       <c r="L233" s="8"/>
     </row>
@@ -9348,7 +9823,9 @@
       <c r="G234" s="3"/>
       <c r="H234" s="4"/>
       <c r="I234" s="4"/>
-      <c r="J234" s="7"/>
+      <c r="J234" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K234" s="8"/>
       <c r="L234" s="8"/>
     </row>
@@ -9372,7 +9849,9 @@
       <c r="G235" s="3"/>
       <c r="H235" s="4"/>
       <c r="I235" s="4"/>
-      <c r="J235" s="7"/>
+      <c r="J235" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K235" s="8"/>
       <c r="L235" s="8"/>
     </row>
@@ -9396,7 +9875,9 @@
       <c r="G236" s="3"/>
       <c r="H236" s="4"/>
       <c r="I236" s="4"/>
-      <c r="J236" s="7"/>
+      <c r="J236" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K236" s="8"/>
       <c r="L236" s="8"/>
     </row>
@@ -9420,7 +9901,9 @@
       <c r="G237" s="3"/>
       <c r="H237" s="4"/>
       <c r="I237" s="4"/>
-      <c r="J237" s="7"/>
+      <c r="J237" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K237" s="8"/>
       <c r="L237" s="8"/>
     </row>
@@ -9444,7 +9927,9 @@
       <c r="G238" s="3"/>
       <c r="H238" s="4"/>
       <c r="I238" s="4"/>
-      <c r="J238" s="7"/>
+      <c r="J238" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K238" s="8"/>
       <c r="L238" s="8"/>
     </row>
@@ -9468,7 +9953,9 @@
       <c r="G239" s="3"/>
       <c r="H239" s="4"/>
       <c r="I239" s="4"/>
-      <c r="J239" s="7"/>
+      <c r="J239" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K239" s="8"/>
       <c r="L239" s="8"/>
     </row>
@@ -9492,7 +9979,9 @@
       <c r="G240" s="3"/>
       <c r="H240" s="4"/>
       <c r="I240" s="4"/>
-      <c r="J240" s="7"/>
+      <c r="J240" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K240" s="8"/>
       <c r="L240" s="8"/>
     </row>
@@ -9516,7 +10005,9 @@
       <c r="G241" s="3"/>
       <c r="H241" s="4"/>
       <c r="I241" s="4"/>
-      <c r="J241" s="7"/>
+      <c r="J241" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K241" s="8"/>
       <c r="L241" s="8"/>
     </row>
@@ -9540,7 +10031,9 @@
       <c r="G242" s="3"/>
       <c r="H242" s="4"/>
       <c r="I242" s="4"/>
-      <c r="J242" s="7"/>
+      <c r="J242" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K242" s="8"/>
       <c r="L242" s="8"/>
     </row>
@@ -9564,7 +10057,9 @@
       <c r="G243" s="3"/>
       <c r="H243" s="4"/>
       <c r="I243" s="4"/>
-      <c r="J243" s="7"/>
+      <c r="J243" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K243" s="8"/>
       <c r="L243" s="8"/>
     </row>
@@ -9588,7 +10083,9 @@
       <c r="G244" s="3"/>
       <c r="H244" s="4"/>
       <c r="I244" s="4"/>
-      <c r="J244" s="7"/>
+      <c r="J244" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K244" s="8"/>
       <c r="L244" s="8"/>
     </row>
@@ -9612,7 +10109,9 @@
       <c r="G245" s="3"/>
       <c r="H245" s="4"/>
       <c r="I245" s="4"/>
-      <c r="J245" s="7"/>
+      <c r="J245" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K245" s="8"/>
       <c r="L245" s="8"/>
     </row>
@@ -9636,7 +10135,9 @@
       <c r="G246" s="3"/>
       <c r="H246" s="4"/>
       <c r="I246" s="4"/>
-      <c r="J246" s="7"/>
+      <c r="J246" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K246" s="8"/>
       <c r="L246" s="8"/>
     </row>
@@ -9660,7 +10161,9 @@
       <c r="G247" s="3"/>
       <c r="H247" s="4"/>
       <c r="I247" s="4"/>
-      <c r="J247" s="7"/>
+      <c r="J247" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K247" s="8"/>
       <c r="L247" s="8"/>
     </row>
@@ -9684,7 +10187,9 @@
       <c r="G248" s="3"/>
       <c r="H248" s="4"/>
       <c r="I248" s="4"/>
-      <c r="J248" s="7"/>
+      <c r="J248" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K248" s="8"/>
       <c r="L248" s="8"/>
     </row>
@@ -9708,7 +10213,9 @@
       <c r="G249" s="3"/>
       <c r="H249" s="4"/>
       <c r="I249" s="4"/>
-      <c r="J249" s="7"/>
+      <c r="J249" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K249" s="8"/>
       <c r="L249" s="8"/>
     </row>
@@ -9732,7 +10239,9 @@
       <c r="G250" s="3"/>
       <c r="H250" s="4"/>
       <c r="I250" s="4"/>
-      <c r="J250" s="7"/>
+      <c r="J250" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K250" s="8"/>
       <c r="L250" s="8"/>
     </row>
@@ -9756,7 +10265,9 @@
       <c r="G251" s="3"/>
       <c r="H251" s="4"/>
       <c r="I251" s="4"/>
-      <c r="J251" s="7"/>
+      <c r="J251" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K251" s="8"/>
       <c r="L251" s="8"/>
     </row>
@@ -9780,7 +10291,9 @@
       <c r="G252" s="3"/>
       <c r="H252" s="4"/>
       <c r="I252" s="4"/>
-      <c r="J252" s="7"/>
+      <c r="J252" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K252" s="8"/>
       <c r="L252" s="8"/>
     </row>
@@ -9804,7 +10317,9 @@
       <c r="G253" s="3"/>
       <c r="H253" s="4"/>
       <c r="I253" s="4"/>
-      <c r="J253" s="7"/>
+      <c r="J253" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K253" s="8"/>
       <c r="L253" s="8"/>
     </row>
@@ -9828,7 +10343,9 @@
       <c r="G254" s="3"/>
       <c r="H254" s="4"/>
       <c r="I254" s="4"/>
-      <c r="J254" s="7"/>
+      <c r="J254" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K254" s="8"/>
       <c r="L254" s="8"/>
     </row>
@@ -9852,7 +10369,9 @@
       <c r="G255" s="3"/>
       <c r="H255" s="4"/>
       <c r="I255" s="4"/>
-      <c r="J255" s="7"/>
+      <c r="J255" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K255" s="8"/>
       <c r="L255" s="8"/>
     </row>
@@ -9876,7 +10395,9 @@
       <c r="G256" s="3"/>
       <c r="H256" s="4"/>
       <c r="I256" s="4"/>
-      <c r="J256" s="7"/>
+      <c r="J256" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K256" s="8"/>
       <c r="L256" s="8"/>
     </row>
@@ -9900,7 +10421,9 @@
       <c r="G257" s="3"/>
       <c r="H257" s="4"/>
       <c r="I257" s="4"/>
-      <c r="J257" s="7"/>
+      <c r="J257" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K257" s="8"/>
       <c r="L257" s="8"/>
     </row>
@@ -9924,7 +10447,9 @@
       <c r="G258" s="3"/>
       <c r="H258" s="4"/>
       <c r="I258" s="4"/>
-      <c r="J258" s="7"/>
+      <c r="J258" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K258" s="8"/>
       <c r="L258" s="8"/>
     </row>
@@ -9948,7 +10473,9 @@
       <c r="G259" s="3"/>
       <c r="H259" s="4"/>
       <c r="I259" s="4"/>
-      <c r="J259" s="7"/>
+      <c r="J259" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K259" s="8"/>
       <c r="L259" s="8"/>
     </row>
@@ -9972,7 +10499,9 @@
       <c r="G260" s="3"/>
       <c r="H260" s="4"/>
       <c r="I260" s="4"/>
-      <c r="J260" s="7"/>
+      <c r="J260" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K260" s="8"/>
       <c r="L260" s="8"/>
     </row>
@@ -9996,7 +10525,9 @@
       <c r="G261" s="3"/>
       <c r="H261" s="4"/>
       <c r="I261" s="4"/>
-      <c r="J261" s="7"/>
+      <c r="J261" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K261" s="8"/>
       <c r="L261" s="8"/>
     </row>
@@ -10020,7 +10551,9 @@
       <c r="G262" s="3"/>
       <c r="H262" s="4"/>
       <c r="I262" s="4"/>
-      <c r="J262" s="7"/>
+      <c r="J262" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K262" s="8"/>
       <c r="L262" s="8"/>
     </row>
@@ -10044,7 +10577,9 @@
       <c r="G263" s="3"/>
       <c r="H263" s="4"/>
       <c r="I263" s="4"/>
-      <c r="J263" s="7"/>
+      <c r="J263" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K263" s="8"/>
       <c r="L263" s="8"/>
     </row>
@@ -10068,7 +10603,9 @@
       <c r="G264" s="3"/>
       <c r="H264" s="4"/>
       <c r="I264" s="4"/>
-      <c r="J264" s="7"/>
+      <c r="J264" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K264" s="8"/>
       <c r="L264" s="8"/>
     </row>
@@ -10092,7 +10629,9 @@
       <c r="G265" s="3"/>
       <c r="H265" s="4"/>
       <c r="I265" s="4"/>
-      <c r="J265" s="7"/>
+      <c r="J265" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K265" s="8"/>
       <c r="L265" s="8"/>
     </row>
@@ -10116,7 +10655,9 @@
       <c r="G266" s="3"/>
       <c r="H266" s="4"/>
       <c r="I266" s="4"/>
-      <c r="J266" s="7"/>
+      <c r="J266" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K266" s="8"/>
       <c r="L266" s="8"/>
     </row>
@@ -10140,7 +10681,9 @@
       <c r="G267" s="3"/>
       <c r="H267" s="4"/>
       <c r="I267" s="4"/>
-      <c r="J267" s="7"/>
+      <c r="J267" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K267" s="8"/>
       <c r="L267" s="8"/>
     </row>
@@ -10164,7 +10707,9 @@
       <c r="G268" s="3"/>
       <c r="H268" s="4"/>
       <c r="I268" s="4"/>
-      <c r="J268" s="7"/>
+      <c r="J268" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K268" s="8"/>
       <c r="L268" s="8"/>
     </row>
@@ -10188,7 +10733,9 @@
       <c r="G269" s="3"/>
       <c r="H269" s="4"/>
       <c r="I269" s="4"/>
-      <c r="J269" s="7"/>
+      <c r="J269" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K269" s="8"/>
       <c r="L269" s="8"/>
     </row>
@@ -10212,7 +10759,9 @@
       <c r="G270" s="3"/>
       <c r="H270" s="4"/>
       <c r="I270" s="4"/>
-      <c r="J270" s="7"/>
+      <c r="J270" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K270" s="8"/>
       <c r="L270" s="8"/>
     </row>
@@ -10236,7 +10785,9 @@
       <c r="G271" s="3"/>
       <c r="H271" s="4"/>
       <c r="I271" s="4"/>
-      <c r="J271" s="7"/>
+      <c r="J271" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K271" s="8"/>
       <c r="L271" s="8"/>
     </row>
@@ -10260,7 +10811,9 @@
       <c r="G272" s="3"/>
       <c r="H272" s="4"/>
       <c r="I272" s="4"/>
-      <c r="J272" s="7"/>
+      <c r="J272" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K272" s="8"/>
       <c r="L272" s="8"/>
     </row>
@@ -10284,7 +10837,9 @@
       <c r="G273" s="3"/>
       <c r="H273" s="4"/>
       <c r="I273" s="4"/>
-      <c r="J273" s="7"/>
+      <c r="J273" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K273" s="8"/>
       <c r="L273" s="8"/>
     </row>
@@ -10308,7 +10863,9 @@
       <c r="G274" s="3"/>
       <c r="H274" s="4"/>
       <c r="I274" s="4"/>
-      <c r="J274" s="7"/>
+      <c r="J274" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K274" s="8"/>
       <c r="L274" s="8"/>
     </row>
@@ -10332,7 +10889,9 @@
       <c r="G275" s="3"/>
       <c r="H275" s="4"/>
       <c r="I275" s="4"/>
-      <c r="J275" s="7"/>
+      <c r="J275" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K275" s="8"/>
       <c r="L275" s="8"/>
     </row>
@@ -10356,7 +10915,9 @@
       <c r="G276" s="3"/>
       <c r="H276" s="4"/>
       <c r="I276" s="4"/>
-      <c r="J276" s="7"/>
+      <c r="J276" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K276" s="8"/>
       <c r="L276" s="8"/>
     </row>
@@ -10380,7 +10941,9 @@
       <c r="G277" s="3"/>
       <c r="H277" s="4"/>
       <c r="I277" s="4"/>
-      <c r="J277" s="7"/>
+      <c r="J277" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K277" s="8"/>
       <c r="L277" s="8"/>
     </row>
@@ -10404,7 +10967,9 @@
       <c r="G278" s="3"/>
       <c r="H278" s="4"/>
       <c r="I278" s="4"/>
-      <c r="J278" s="7"/>
+      <c r="J278" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K278" s="8"/>
       <c r="L278" s="8"/>
     </row>
@@ -10428,7 +10993,9 @@
       <c r="G279" s="3"/>
       <c r="H279" s="4"/>
       <c r="I279" s="4"/>
-      <c r="J279" s="7"/>
+      <c r="J279" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K279" s="8"/>
       <c r="L279" s="8"/>
     </row>
@@ -10452,7 +11019,9 @@
       <c r="G280" s="3"/>
       <c r="H280" s="4"/>
       <c r="I280" s="4"/>
-      <c r="J280" s="7"/>
+      <c r="J280" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K280" s="8"/>
       <c r="L280" s="8"/>
     </row>
@@ -10476,7 +11045,9 @@
       <c r="G281" s="3"/>
       <c r="H281" s="4"/>
       <c r="I281" s="4"/>
-      <c r="J281" s="7"/>
+      <c r="J281" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K281" s="8"/>
       <c r="L281" s="8"/>
     </row>
@@ -10500,7 +11071,9 @@
       <c r="G282" s="3"/>
       <c r="H282" s="4"/>
       <c r="I282" s="4"/>
-      <c r="J282" s="7"/>
+      <c r="J282" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K282" s="8"/>
       <c r="L282" s="8"/>
     </row>
@@ -10524,7 +11097,9 @@
       <c r="G283" s="3"/>
       <c r="H283" s="4"/>
       <c r="I283" s="4"/>
-      <c r="J283" s="7"/>
+      <c r="J283" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K283" s="8"/>
       <c r="L283" s="8"/>
     </row>
@@ -10548,7 +11123,9 @@
       <c r="G284" s="3"/>
       <c r="H284" s="4"/>
       <c r="I284" s="4"/>
-      <c r="J284" s="7"/>
+      <c r="J284" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K284" s="8"/>
       <c r="L284" s="8"/>
     </row>
@@ -10572,7 +11149,9 @@
       <c r="G285" s="3"/>
       <c r="H285" s="4"/>
       <c r="I285" s="4"/>
-      <c r="J285" s="7"/>
+      <c r="J285" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K285" s="8"/>
       <c r="L285" s="8"/>
     </row>
@@ -10596,7 +11175,9 @@
       <c r="G286" s="3"/>
       <c r="H286" s="4"/>
       <c r="I286" s="4"/>
-      <c r="J286" s="7"/>
+      <c r="J286" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K286" s="8"/>
       <c r="L286" s="8"/>
     </row>
@@ -10620,7 +11201,9 @@
       <c r="G287" s="3"/>
       <c r="H287" s="4"/>
       <c r="I287" s="4"/>
-      <c r="J287" s="7"/>
+      <c r="J287" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K287" s="8"/>
       <c r="L287" s="8"/>
     </row>
@@ -10644,7 +11227,9 @@
       <c r="G288" s="3"/>
       <c r="H288" s="4"/>
       <c r="I288" s="4"/>
-      <c r="J288" s="7"/>
+      <c r="J288" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K288" s="8"/>
       <c r="L288" s="8"/>
     </row>
@@ -10668,7 +11253,9 @@
       <c r="G289" s="3"/>
       <c r="H289" s="4"/>
       <c r="I289" s="4"/>
-      <c r="J289" s="7"/>
+      <c r="J289" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K289" s="8"/>
       <c r="L289" s="8"/>
     </row>
@@ -10692,7 +11279,9 @@
       <c r="G290" s="3"/>
       <c r="H290" s="4"/>
       <c r="I290" s="4"/>
-      <c r="J290" s="7"/>
+      <c r="J290" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K290" s="8"/>
       <c r="L290" s="8"/>
     </row>
@@ -10716,7 +11305,9 @@
       <c r="G291" s="3"/>
       <c r="H291" s="4"/>
       <c r="I291" s="4"/>
-      <c r="J291" s="7"/>
+      <c r="J291" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K291" s="8"/>
       <c r="L291" s="8"/>
     </row>
@@ -10740,7 +11331,9 @@
       <c r="G292" s="3"/>
       <c r="H292" s="4"/>
       <c r="I292" s="4"/>
-      <c r="J292" s="7"/>
+      <c r="J292" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K292" s="8"/>
       <c r="L292" s="8"/>
     </row>
@@ -10764,7 +11357,9 @@
       <c r="G293" s="3"/>
       <c r="H293" s="4"/>
       <c r="I293" s="4"/>
-      <c r="J293" s="7"/>
+      <c r="J293" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K293" s="8"/>
       <c r="L293" s="8"/>
     </row>
@@ -10788,7 +11383,9 @@
       <c r="G294" s="3"/>
       <c r="H294" s="4"/>
       <c r="I294" s="4"/>
-      <c r="J294" s="7"/>
+      <c r="J294" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K294" s="8"/>
       <c r="L294" s="8"/>
     </row>
@@ -10812,7 +11409,9 @@
       <c r="G295" s="3"/>
       <c r="H295" s="4"/>
       <c r="I295" s="4"/>
-      <c r="J295" s="7"/>
+      <c r="J295" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K295" s="8"/>
       <c r="L295" s="8"/>
     </row>
@@ -10836,7 +11435,9 @@
       <c r="G296" s="3"/>
       <c r="H296" s="4"/>
       <c r="I296" s="4"/>
-      <c r="J296" s="7"/>
+      <c r="J296" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K296" s="8"/>
       <c r="L296" s="8"/>
     </row>
@@ -10860,7 +11461,9 @@
       <c r="G297" s="3"/>
       <c r="H297" s="4"/>
       <c r="I297" s="4"/>
-      <c r="J297" s="7"/>
+      <c r="J297" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K297" s="8"/>
       <c r="L297" s="8"/>
     </row>
@@ -10884,7 +11487,9 @@
       <c r="G298" s="3"/>
       <c r="H298" s="4"/>
       <c r="I298" s="4"/>
-      <c r="J298" s="7"/>
+      <c r="J298" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K298" s="8"/>
       <c r="L298" s="8"/>
     </row>
@@ -10908,7 +11513,9 @@
       <c r="G299" s="3"/>
       <c r="H299" s="4"/>
       <c r="I299" s="4"/>
-      <c r="J299" s="7"/>
+      <c r="J299" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K299" s="8"/>
       <c r="L299" s="8"/>
     </row>
@@ -10934,7 +11541,9 @@
       <c r="I300" s="10" t="s">
         <v>432</v>
       </c>
-      <c r="J300" s="7"/>
+      <c r="J300" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K300" s="8"/>
       <c r="L300" s="8"/>
     </row>
@@ -10958,7 +11567,9 @@
       <c r="G301" s="3"/>
       <c r="H301" s="4"/>
       <c r="I301" s="4"/>
-      <c r="J301" s="7"/>
+      <c r="J301" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K301" s="8"/>
       <c r="L301" s="8"/>
     </row>
@@ -10982,7 +11593,9 @@
       <c r="G302" s="3"/>
       <c r="H302" s="4"/>
       <c r="I302" s="4"/>
-      <c r="J302" s="7"/>
+      <c r="J302" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K302" s="8"/>
       <c r="L302" s="8"/>
     </row>
@@ -11006,7 +11619,9 @@
       <c r="G303" s="3"/>
       <c r="H303" s="4"/>
       <c r="I303" s="4"/>
-      <c r="J303" s="7"/>
+      <c r="J303" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K303" s="8"/>
       <c r="L303" s="8"/>
     </row>
@@ -11030,7 +11645,9 @@
       <c r="G304" s="3"/>
       <c r="H304" s="4"/>
       <c r="I304" s="4"/>
-      <c r="J304" s="7"/>
+      <c r="J304" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K304" s="8"/>
       <c r="L304" s="8"/>
     </row>
@@ -11054,7 +11671,9 @@
       <c r="G305" s="3"/>
       <c r="H305" s="4"/>
       <c r="I305" s="4"/>
-      <c r="J305" s="7"/>
+      <c r="J305" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K305" s="8"/>
       <c r="L305" s="8"/>
     </row>
@@ -11078,7 +11697,9 @@
       <c r="G306" s="3"/>
       <c r="H306" s="4"/>
       <c r="I306" s="4"/>
-      <c r="J306" s="7"/>
+      <c r="J306" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K306" s="8"/>
       <c r="L306" s="8"/>
     </row>
@@ -11102,7 +11723,9 @@
       <c r="G307" s="3"/>
       <c r="H307" s="4"/>
       <c r="I307" s="4"/>
-      <c r="J307" s="7"/>
+      <c r="J307" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K307" s="8"/>
       <c r="L307" s="8"/>
     </row>
@@ -11126,7 +11749,9 @@
       <c r="G308" s="3"/>
       <c r="H308" s="4"/>
       <c r="I308" s="4"/>
-      <c r="J308" s="7"/>
+      <c r="J308" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K308" s="8"/>
       <c r="L308" s="8"/>
     </row>
@@ -11150,7 +11775,9 @@
       <c r="G309" s="3"/>
       <c r="H309" s="4"/>
       <c r="I309" s="4"/>
-      <c r="J309" s="7"/>
+      <c r="J309" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K309" s="8"/>
       <c r="L309" s="8"/>
     </row>
@@ -11174,7 +11801,9 @@
       <c r="G310" s="3"/>
       <c r="H310" s="4"/>
       <c r="I310" s="4"/>
-      <c r="J310" s="7"/>
+      <c r="J310" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K310" s="8"/>
       <c r="L310" s="8"/>
     </row>
@@ -11198,7 +11827,9 @@
       <c r="G311" s="3"/>
       <c r="H311" s="4"/>
       <c r="I311" s="4"/>
-      <c r="J311" s="7"/>
+      <c r="J311" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K311" s="8"/>
       <c r="L311" s="8"/>
     </row>
@@ -11222,7 +11853,9 @@
       <c r="G312" s="3"/>
       <c r="H312" s="4"/>
       <c r="I312" s="4"/>
-      <c r="J312" s="7"/>
+      <c r="J312" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K312" s="8"/>
       <c r="L312" s="8"/>
     </row>
@@ -11246,7 +11879,9 @@
       <c r="G313" s="3"/>
       <c r="H313" s="4"/>
       <c r="I313" s="4"/>
-      <c r="J313" s="7"/>
+      <c r="J313" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K313" s="8"/>
       <c r="L313" s="8"/>
     </row>
@@ -11270,7 +11905,9 @@
       <c r="G314" s="3"/>
       <c r="H314" s="4"/>
       <c r="I314" s="4"/>
-      <c r="J314" s="7"/>
+      <c r="J314" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K314" s="8"/>
       <c r="L314" s="8"/>
     </row>
@@ -11294,7 +11931,9 @@
       <c r="G315" s="3"/>
       <c r="H315" s="4"/>
       <c r="I315" s="4"/>
-      <c r="J315" s="7"/>
+      <c r="J315" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K315" s="8"/>
       <c r="L315" s="8"/>
     </row>
@@ -11318,7 +11957,9 @@
       <c r="G316" s="3"/>
       <c r="H316" s="4"/>
       <c r="I316" s="4"/>
-      <c r="J316" s="7"/>
+      <c r="J316" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K316" s="8"/>
       <c r="L316" s="8"/>
     </row>
@@ -11346,7 +11987,9 @@
         <v>917</v>
       </c>
       <c r="I317" s="4"/>
-      <c r="J317" s="7"/>
+      <c r="J317" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K317" s="8"/>
       <c r="L317" s="8"/>
     </row>
@@ -11370,7 +12013,9 @@
       <c r="G318" s="3"/>
       <c r="H318" s="4"/>
       <c r="I318" s="4"/>
-      <c r="J318" s="7"/>
+      <c r="J318" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K318" s="8"/>
       <c r="L318" s="8"/>
     </row>
@@ -11400,7 +12045,9 @@
       <c r="I319" s="10" t="s">
         <v>923</v>
       </c>
-      <c r="J319" s="7"/>
+      <c r="J319" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K319" s="8"/>
       <c r="L319" s="8"/>
     </row>
@@ -11424,7 +12071,9 @@
       <c r="G320" s="3"/>
       <c r="H320" s="4"/>
       <c r="I320" s="4"/>
-      <c r="J320" s="7"/>
+      <c r="J320" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K320" s="8"/>
       <c r="L320" s="8"/>
     </row>
@@ -11448,7 +12097,9 @@
       <c r="G321" s="3"/>
       <c r="H321" s="4"/>
       <c r="I321" s="4"/>
-      <c r="J321" s="7"/>
+      <c r="J321" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K321" s="8"/>
       <c r="L321" s="8"/>
     </row>
@@ -11472,7 +12123,9 @@
       <c r="G322" s="3"/>
       <c r="H322" s="4"/>
       <c r="I322" s="4"/>
-      <c r="J322" s="7"/>
+      <c r="J322" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K322" s="8"/>
       <c r="L322" s="8"/>
     </row>
@@ -11496,7 +12149,9 @@
       <c r="G323" s="3"/>
       <c r="H323" s="4"/>
       <c r="I323" s="4"/>
-      <c r="J323" s="7"/>
+      <c r="J323" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K323" s="8"/>
       <c r="L323" s="8"/>
     </row>
@@ -11520,7 +12175,9 @@
       <c r="G324" s="3"/>
       <c r="H324" s="4"/>
       <c r="I324" s="4"/>
-      <c r="J324" s="7"/>
+      <c r="J324" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K324" s="8"/>
       <c r="L324" s="8"/>
     </row>
@@ -11544,7 +12201,9 @@
       <c r="G325" s="3"/>
       <c r="H325" s="4"/>
       <c r="I325" s="4"/>
-      <c r="J325" s="7"/>
+      <c r="J325" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K325" s="8"/>
       <c r="L325" s="8"/>
     </row>
@@ -11568,7 +12227,9 @@
       <c r="G326" s="3"/>
       <c r="H326" s="4"/>
       <c r="I326" s="4"/>
-      <c r="J326" s="7"/>
+      <c r="J326" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K326" s="8"/>
       <c r="L326" s="8"/>
     </row>
@@ -11592,7 +12253,9 @@
       <c r="G327" s="3"/>
       <c r="H327" s="4"/>
       <c r="I327" s="4"/>
-      <c r="J327" s="7"/>
+      <c r="J327" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K327" s="8"/>
       <c r="L327" s="8"/>
     </row>
@@ -11616,7 +12279,9 @@
       <c r="G328" s="3"/>
       <c r="H328" s="4"/>
       <c r="I328" s="4"/>
-      <c r="J328" s="7"/>
+      <c r="J328" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K328" s="8"/>
       <c r="L328" s="8"/>
     </row>
@@ -11640,7 +12305,9 @@
       <c r="G329" s="3"/>
       <c r="H329" s="4"/>
       <c r="I329" s="4"/>
-      <c r="J329" s="7"/>
+      <c r="J329" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K329" s="8"/>
       <c r="L329" s="8"/>
     </row>
@@ -11664,7 +12331,9 @@
       <c r="G330" s="3"/>
       <c r="H330" s="4"/>
       <c r="I330" s="4"/>
-      <c r="J330" s="7"/>
+      <c r="J330" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K330" s="8"/>
       <c r="L330" s="8"/>
     </row>
@@ -11688,7 +12357,9 @@
       <c r="G331" s="3"/>
       <c r="H331" s="4"/>
       <c r="I331" s="4"/>
-      <c r="J331" s="7"/>
+      <c r="J331" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K331" s="8"/>
       <c r="L331" s="8"/>
     </row>
@@ -11712,7 +12383,9 @@
       <c r="G332" s="3"/>
       <c r="H332" s="4"/>
       <c r="I332" s="4"/>
-      <c r="J332" s="7"/>
+      <c r="J332" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K332" s="8"/>
       <c r="L332" s="8"/>
     </row>
@@ -11736,7 +12409,9 @@
       <c r="G333" s="3"/>
       <c r="H333" s="4"/>
       <c r="I333" s="4"/>
-      <c r="J333" s="7"/>
+      <c r="J333" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K333" s="8"/>
       <c r="L333" s="8"/>
     </row>
@@ -11760,7 +12435,9 @@
       <c r="G334" s="3"/>
       <c r="H334" s="4"/>
       <c r="I334" s="4"/>
-      <c r="J334" s="7"/>
+      <c r="J334" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K334" s="8"/>
       <c r="L334" s="8"/>
     </row>
@@ -11784,7 +12461,9 @@
       <c r="G335" s="3"/>
       <c r="H335" s="4"/>
       <c r="I335" s="4"/>
-      <c r="J335" s="7"/>
+      <c r="J335" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K335" s="8"/>
       <c r="L335" s="8"/>
     </row>
@@ -11808,7 +12487,9 @@
       <c r="G336" s="3"/>
       <c r="H336" s="4"/>
       <c r="I336" s="4"/>
-      <c r="J336" s="7"/>
+      <c r="J336" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K336" s="8"/>
       <c r="L336" s="8"/>
     </row>
@@ -11832,7 +12513,9 @@
       <c r="G337" s="3"/>
       <c r="H337" s="4"/>
       <c r="I337" s="4"/>
-      <c r="J337" s="7"/>
+      <c r="J337" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K337" s="8"/>
       <c r="L337" s="8"/>
     </row>
@@ -11856,7 +12539,9 @@
       <c r="G338" s="3"/>
       <c r="H338" s="4"/>
       <c r="I338" s="4"/>
-      <c r="J338" s="7"/>
+      <c r="J338" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K338" s="8"/>
       <c r="L338" s="8"/>
     </row>
@@ -11880,7 +12565,9 @@
       <c r="G339" s="3"/>
       <c r="H339" s="4"/>
       <c r="I339" s="4"/>
-      <c r="J339" s="7"/>
+      <c r="J339" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K339" s="8"/>
       <c r="L339" s="8"/>
     </row>
@@ -11904,7 +12591,9 @@
       <c r="G340" s="3"/>
       <c r="H340" s="4"/>
       <c r="I340" s="4"/>
-      <c r="J340" s="7"/>
+      <c r="J340" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K340" s="8"/>
       <c r="L340" s="8"/>
     </row>
@@ -11928,7 +12617,9 @@
       <c r="G341" s="3"/>
       <c r="H341" s="4"/>
       <c r="I341" s="4"/>
-      <c r="J341" s="7"/>
+      <c r="J341" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K341" s="8"/>
       <c r="L341" s="8"/>
     </row>
@@ -11952,7 +12643,9 @@
       <c r="G342" s="3"/>
       <c r="H342" s="4"/>
       <c r="I342" s="4"/>
-      <c r="J342" s="7"/>
+      <c r="J342" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K342" s="8"/>
       <c r="L342" s="8"/>
     </row>
@@ -11976,14 +12669,19 @@
       <c r="G343" s="3"/>
       <c r="H343" s="4"/>
       <c r="I343" s="4"/>
-      <c r="J343" s="7"/>
+      <c r="J343" s="7" t="s">
+        <v>988</v>
+      </c>
       <c r="K343" s="8"/>
       <c r="L343" s="8"/>
+    </row>
+    <row r="1048576" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J1048576" s="7"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L343" xr:uid="{E8848DF5-3B9B-4C93-95E8-BF114BFDF30F}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J343" xr:uid="{8B475F9E-93A8-4435-A686-0C2051F11A82}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J1048576 J2:J343" xr:uid="{8B475F9E-93A8-4435-A686-0C2051F11A82}">
       <formula1>"OK,Use my Spanish,Keep current,Discuss"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>